<commit_message>
11 05 2024 get screener df into the execute strategy client. must next build out execute strategy to take stream and figure out fastest way to read and act based on stream.
</commit_message>
<xml_diff>
--- a/screener/daily_screener_signals/2024-11-06.xlsx
+++ b/screener/daily_screener_signals/2024-11-06.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>222.9840523612365</v>
       </c>
       <c r="K2" t="n">
         <v>4.994145044040784</v>
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>148.3652916128462</v>
       </c>
       <c r="K3" t="n">
         <v>7.505897692742969</v>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>6.774944128546786</v>
       </c>
       <c r="K4" t="n">
         <v>164.372528964142</v>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>200.3140617619091</v>
       </c>
       <c r="K5" t="n">
         <v>5.559343613748041</v>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>406.5521510422566</v>
       </c>
       <c r="K6" t="n">
         <v>2.739168141516615</v>
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>2749.116186350202</v>
       </c>
       <c r="K7" t="n">
         <v>0.4050809876749749</v>
@@ -1006,7 +1006,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>198.4121640776024</v>
       </c>
       <c r="K8" t="n">
         <v>5.612633203095583</v>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>4.245669745949531</v>
       </c>
       <c r="K9" t="n">
         <v>262.2942354530554</v>
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>279.7940102441034</v>
       </c>
       <c r="K10" t="n">
         <v>3.980123445203271</v>
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>8554.793297911887</v>
       </c>
       <c r="K11" t="n">
         <v>0.1301743550334312</v>
@@ -1302,7 +1302,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>43.33205821111165</v>
       </c>
       <c r="K12" t="n">
         <v>25.69955700175893</v>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>20637.32999722507</v>
       </c>
       <c r="K13" t="n">
         <v>0.05396118103212666</v>
@@ -1450,7 +1450,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>340.4956316265796</v>
       </c>
       <c r="K14" t="n">
         <v>3.270569712392956</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>2252.473234635582</v>
       </c>
       <c r="K15" t="n">
         <v>0.4943964185129006</v>
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>914.5611855736092</v>
       </c>
       <c r="K16" t="n">
         <v>1.217649204412218</v>

</xml_diff>